<commit_message>
Committing Generated Files 43
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads with correct URL and required controls</t>
+          <t>Verify login page loads with correct URL and UI elements</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -488,12 +488,12 @@
         <is>
           <t>Open a browser
 Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the loaded page</t>
+Observe the page URL and login form elements</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads successfully, browser URL remains http://172.21.166.115/washtabui/login?data=undefined, and username textbox, password textbox, SIGN IN button, home button, and arrow back button are visible.</t>
+          <t>Browser URL remains http://172.21.166.115/washtabui/login?data=undefined and username textbox, password textbox, SIGN IN button, home navigation button, and back navigation button are visible on the page</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify login page input fields accept user input</t>
+          <t>Verify username textbox is visible and accepts input</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,16 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the username textbox
-Type any text value
-Click the password textbox
-Type any password value</t>
+          <t>Open the login page URL
+Locate the username textbox
+Click inside the username textbox and type a sample username</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Username textbox accepts typed input and displays entered text. Password textbox accepts input and displays masked characters.</t>
+          <t>Username textbox is visible, enabled, receives focus when clicked, and displays the entered text</t>
         </is>
       </c>
     </row>
@@ -542,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify successful login with valid credentials</t>
+          <t>Verify password textbox is visible and masks characters</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,15 +556,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr into the username textbox
-Enter Icstunnel1 into the password textbox
-Click the SIGN IN button</t>
+          <t>Open the login page URL
+Locate the password textbox
+Type a sample password into the password textbox</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>User is authenticated successfully and the application redirects to the home page with URL http://172.21.166.115/washtabui/home. Login page is no longer displayed.</t>
+          <t>Password textbox is visible and enabled and the entered characters are masked (shown as dots or asterisks) instead of plain text</t>
         </is>
       </c>
     </row>
@@ -578,12 +575,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect password</t>
+          <t>Verify SIGN IN button is visible and clickable</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -594,15 +591,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr into the username textbox
-Enter IncorrectPassword into the password textbox
-Click the SIGN IN button</t>
+          <t>Open the login page URL
+Locate the SIGN IN button
+Click the SIGN IN button without entering credentials</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication fails and the user remains on the login page. Browser URL stays http://172.21.166.115/washtabui/login?data=undefined and access to the home page is not granted.</t>
+          <t>SIGN IN button is visible and clickable and the login form remains on the login page indicating login cannot proceed without valid credentials</t>
         </is>
       </c>
     </row>
@@ -614,12 +610,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect username</t>
+          <t>Verify successful login with valid credentials</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -630,15 +626,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter invaliduser into the username textbox
-Enter Icstunnel1 into the password textbox
+          <t>Open the login page URL
+Enter hacklarr in the username textbox
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails and the application remains on the login page without redirecting to the home page.</t>
+          <t>User is authenticated successfully and redirected to the home page where the browser URL becomes http://172.21.166.115/washtabui/home and the home page UI is displayed</t>
         </is>
       </c>
     </row>
@@ -650,7 +646,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify login fails when both username and password are incorrect</t>
+          <t>Verify login fails with incorrect password</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -666,15 +662,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter wronguser into the username textbox
-Enter wrongpassword into the password textbox
+          <t>Open the login page URL
+Enter hacklarr in the username textbox
+Enter incorrectPassword in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication is rejected and the application keeps the user on the login page without navigation to the home page.</t>
+          <t>Authentication fails, user remains on the login page URL, the application does not navigate to the home page, and a visible authentication failure or sign‑in error message is displayed</t>
         </is>
       </c>
     </row>
@@ -686,7 +682,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify login attempt when username field is empty</t>
+          <t>Verify login fails with invalid username</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -702,15 +698,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the login page
-Leave the username textbox empty
-Enter Icstunnel1 into the password textbox
+          <t>Open the login page URL
+Enter invaliduser in the username textbox
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Login is not completed and the user remains on the login page without being redirected to the home page.</t>
+          <t>Authentication fails and the application remains on the login page without redirecting to the home page and an authentication failure indication is visible</t>
         </is>
       </c>
     </row>
@@ -722,7 +718,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login attempt when password field is empty</t>
+          <t>Verify login fails with both username and password invalid</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -738,15 +734,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr into the username textbox
-Leave the password textbox empty
+          <t>Open the login page URL
+Enter invaliduser in the username textbox
+Enter invalidPassword in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication is not successful and the user remains on the login page without redirection to the home page.</t>
+          <t>Authentication is rejected, the login page remains displayed, and no navigation to http://172.21.166.115/washtabui/home occurs</t>
         </is>
       </c>
     </row>
@@ -758,7 +754,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify login attempt when both username and password fields are empty</t>
+          <t>Verify login attempt with empty username and password</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -774,7 +770,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the login page
+          <t>Open the login page URL
 Leave the username textbox empty
 Leave the password textbox empty
 Click the SIGN IN button</t>
@@ -782,7 +778,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Login attempt is rejected and the application remains on the login page without redirecting to the home page.</t>
+          <t>Login is rejected and the user remains on the login page without navigation to the home page</t>
         </is>
       </c>
     </row>
@@ -794,12 +790,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Verify login attempt with username only</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -810,14 +806,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the password textbox
-Enter any password value</t>
+          <t>Open the login page URL
+Enter hacklarr in the username textbox
+Leave the password textbox empty
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Characters entered in the password textbox are masked and not displayed as plain text.</t>
+          <t>Authentication does not succeed and the application stays on the login page without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -829,12 +826,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify navigation to home page using home button</t>
+          <t>Verify login attempt with password only</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -845,13 +842,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the home button</t>
+          <t>Open the login page URL
+Leave the username textbox empty
+Enter Icstunnel1 in the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Application navigates to the home page and the browser URL becomes http://172.21.166.115/washtabui/home.</t>
+          <t>Authentication does not succeed and the login page remains displayed without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -863,7 +862,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify navigation to home page using back button</t>
+          <t>Verify navigation using home navigation button</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -879,13 +878,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the arrow back button</t>
+          <t>Open the login page URL
+Click the home navigation button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Application navigates to the home page and the browser URL becomes http://172.21.166.115/washtabui/home.</t>
+          <t>Application navigates to the home page and the browser URL becomes http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -897,12 +896,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login submission using Enter key</t>
+          <t>Verify navigation using back navigation button</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -913,195 +912,229 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the login page
+          <t>Open the login page URL
+Click the back navigation button</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Application navigates to the home page and the browser URL becomes http://172.21.166.115/washtabui/home</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WT-LOGIN14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Verify login with leading and trailing whitespace in username</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Open the login page URL
+Enter ' hacklarr ' including leading and trailing spaces in the username textbox
+Enter Icstunnel1 in the password textbox
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Application processes the input without UI errors; user is either authenticated and redirected to the home page if whitespace is trimmed or login fails and the login page remains displayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT-LOGIN15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Verify login with very long username input</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Open the login page URL
+Enter a very long string exceeding typical username length in the username textbox
+Enter Icstunnel1 in the password textbox
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Application handles the long input without crashing or breaking the UI and authentication fails while remaining on the login page</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-LOGIN16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify repeated clicking of SIGN IN button during login attempt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Open the login page URL
 Enter hacklarr in the username textbox
 Enter Icstunnel1 in the password textbox
-Press the Enter key on the keyboard</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Login request is submitted and user is authenticated successfully with redirection to http://172.21.166.115/washtabui/home.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>WT-LOGIN14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Verify login attempt with leading and trailing spaces in username</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+Rapidly click the SIGN IN button multiple times</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Application processes the login request once and redirects to the home page a single time without duplicate redirects or UI errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT-LOGIN17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Verify login submission using Enter key</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter '  hacklarr  ' including leading and trailing spaces in the username textbox
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Open the login page URL
+Enter hacklarr in the username textbox
+Enter Icstunnel1 in the password textbox
+Press the Enter key while focused on the password textbox</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Login form submits and the user is redirected to the home page with URL http://172.21.166.115/washtabui/home</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-LOGIN18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Verify login using pasted credentials</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Open the login page URL
+Paste hacklarr into the username textbox
+Paste Icstunnel1 into the password textbox
+Click the SIGN IN button</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Application accepts pasted values and authenticates successfully and redirects to http://172.21.166.115/washtabui/home</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WT-LOGIN19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Verify username case sensitivity during login</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Open the login page URL
+Enter HACKLARR in the username textbox
 Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Entered value including spaces is submitted. If it does not match the stored username exactly, authentication fails and the user remains on the login page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WT-LOGIN15</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Verify login attempt with whitespace-only values</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter only spaces in the username textbox
-Enter only spaces in the password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Authentication fails and the application remains on the login page without redirecting to the home page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-LOGIN16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Verify system behavior when clicking SIGN IN multiple times rapidly</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter hacklarr into the username textbox
-Enter Icstunnel1 into the password textbox
-Click the SIGN IN button multiple times quickly</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Only one authentication request is processed and the user is redirected once to http://172.21.166.115/washtabui/home without duplicate navigation or application errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>WT-LOGIN17</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Verify login attempt using extremely long username and password values</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter a very long string in the username textbox
-Enter a very long string in the password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Login attempt is rejected or handled safely and the application remains stable while keeping the user on the login page without redirecting to the home page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-LOGIN18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Verify login with copied and pasted credentials</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Open the login page
-Copy hacklarr and paste it into the username textbox
-Copy Icstunnel1 and paste it into the password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Credentials entered via copy and paste are accepted and the user is successfully redirected to http://172.21.166.115/washtabui/home.</t>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>If the system enforces case sensitivity login fails and the user remains on the login page with an authentication error; otherwise the user is redirected to the home page</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 47
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads with all required UI elements</t>
+          <t>Verify login page loads and all required UI elements are visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,18 +486,13 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open browser and navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page layout
-Verify the username textbox is visible
-Verify the password textbox is visible
-Verify the SIGN IN button is visible
-Verify the home navigation button is visible
-Verify the back navigation button is visible</t>
+          <t>Open a browser and navigate to http://172.21.166.115/washtabui/login?data=undefined
+Observe the login page layout and visible controls</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads at the specified URL and the username textbox, password textbox, SIGN IN button, home navigation button, and back navigation button are visible and enabled for interaction.</t>
+          <t>Login page loads successfully with URL http://172.21.166.115/washtabui/login?data=undefined and the username textbox, password textbox, SIGN IN button, home navigation button, and back navigation button are visible and interactable.</t>
         </is>
       </c>
     </row>
@@ -509,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify successful login with valid credentials</t>
+          <t>Verify successful login using valid credentials via SIGN IN button</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,15 +520,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr in username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter hacklarr in the username textbox
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User authentication succeeds and the browser redirects to http://172.21.166.115/washtabui/home where the home page is displayed, confirming an authenticated session.</t>
+          <t>User is authenticated successfully and the application redirects to the home page. Browser URL changes to http://172.21.166.115/washtabui/home and login page elements are no longer visible.</t>
         </is>
       </c>
     </row>
@@ -545,12 +540,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect password</t>
+          <t>Verify login submission using keyboard Enter key after entering valid credentials</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -561,15 +556,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr in username textbox
-Enter WrongPassword123 in password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Enter hacklarr in the username textbox
+Enter Icstunnel1 in the password textbox
+Press Enter on the keyboard while the cursor focus is inside the password textbox</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Authentication fails, the browser remains on the login page URL, and a visible sign-in failure message indicating invalid or incorrect credentials is displayed.</t>
+          <t>Login form is submitted through the keyboard action and the application redirects to the home page with URL http://172.21.166.115/washtabui/home indicating successful authentication.</t>
         </is>
       </c>
     </row>
@@ -581,7 +576,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect username</t>
+          <t>Verify login fails with valid username and incorrect password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -597,15 +592,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter invaliduser in username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter hacklarr in the username textbox
+Enter Icstunnel2 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication fails and the application remains on the login page without redirecting to the home page, displaying a visible authentication failure message.</t>
+          <t>Authentication fails and the user remains on the login page with URL http://172.21.166.115/washtabui/login?data=undefined. A visible sign-in failure or error indication is displayed and the application does not navigate to the home page.</t>
         </is>
       </c>
     </row>
@@ -617,7 +612,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify login fails when both username and password are incorrect</t>
+          <t>Verify login fails with invalid username and valid password</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -633,15 +628,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter wronguser in username textbox
-Enter wrongpassword in password textbox
+          <t>Navigate to the login page
+Enter hacklarr123 in the username textbox
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails, the user remains on the login page, and a visible error message indicates that the credentials are invalid.</t>
+          <t>Authentication is rejected and the application remains on the login page. Browser URL does not change to the home page and a visible login failure indication appears.</t>
         </is>
       </c>
     </row>
@@ -653,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify login validation when username field is empty</t>
+          <t>Verify login fails when both username and password are invalid</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,15 +664,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the login page
-Leave username textbox empty
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter invaliduser in the username textbox
+Enter invalidpass in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Login is rejected, the application remains on the login page, and a visible validation or authentication failure message appears due to missing username.</t>
+          <t>System rejects the authentication attempt and the login page remains visible. Browser URL remains the login URL and a visible authentication failure indication is displayed.</t>
         </is>
       </c>
     </row>
@@ -689,7 +684,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify login validation when password field is empty</t>
+          <t>Verify login attempt when username is empty and password is provided</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -705,15 +700,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr in username textbox
-Leave password textbox empty
+          <t>Navigate to the login page
+Leave the username textbox empty
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Login is rejected, the user remains on the login page, and a visible validation or authentication failure message indicates that the password is missing.</t>
+          <t>Authentication does not succeed and the application remains on the login page with a visible validation or authentication failure indication. No navigation to the home page occurs.</t>
         </is>
       </c>
     </row>
@@ -725,7 +720,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login validation when both username and password are empty</t>
+          <t>Verify login attempt when password is empty and username is provided</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -741,15 +736,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the login page
-Leave username textbox empty
-Leave password textbox empty
+          <t>Navigate to the login page
+Enter hacklarr in the username textbox
+Leave the password textbox empty
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication is not completed and the login page remains displayed with visible feedback indicating that credentials are required.</t>
+          <t>Authentication is rejected and the user remains on the login page. A visible validation or authentication failure indication appears and the browser does not redirect to the home page.</t>
         </is>
       </c>
     </row>
@@ -761,12 +756,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify password textbox masks entered characters</t>
+          <t>Verify login attempt when both username and password fields are empty</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -777,14 +772,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the password textbox
-Enter Icstunnel1 in the password textbox</t>
+          <t>Navigate to the login page
+Leave the username textbox empty
+Leave the password textbox empty
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The password characters are masked (for example with dots or asterisks) and the actual text entered is not visible in plain text.</t>
+          <t>Login submission is rejected and the login page remains visible with a validation or authentication failure indication. Browser does not navigate to the home page.</t>
         </is>
       </c>
     </row>
@@ -796,7 +792,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify navigation to home page using home navigation button</t>
+          <t>Verify password textbox masks entered characters</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -812,13 +808,14 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the home navigation button</t>
+          <t>Navigate to the login page
+Click inside the password textbox
+Type Icstunnel1 into the password textbox</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application navigates from the login page to http://172.21.166.115/washtabui/home and the home page becomes visible.</t>
+          <t>Password characters are not displayed as plain text. Each entered character appears masked (for example as dots or asterisks) confirming the field behaves as a password field.</t>
         </is>
       </c>
     </row>
@@ -830,7 +827,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify navigation to home page using back navigation button</t>
+          <t>Verify navigation to home page using home navigation button from login page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -846,13 +843,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the back navigation button</t>
+          <t>Navigate to the login page
+Click the home navigation button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application navigates away from the login page and loads the home page at http://172.21.166.115/washtabui/home.</t>
+          <t>Application navigates away from the login page and loads the home page. Browser URL becomes http://172.21.166.115/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -864,12 +861,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify username textbox accepts pasted input</t>
+          <t>Verify navigation to home page using back navigation button from login page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -880,16 +877,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Copy the text hacklarr to clipboard
-Open the login page
-Paste the copied value into the username textbox
-Enter Icstunnel1 in password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Click the back navigation button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The pasted value appears correctly in the username textbox and login succeeds, redirecting the user to the home page.</t>
+          <t>Application navigates away from the login page and loads the home page. Browser URL changes to http://172.21.166.115/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -901,7 +895,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login attempt with leading and trailing spaces in username</t>
+          <t>Verify login behavior when credentials contain leading and trailing whitespace</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -917,15 +911,15 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter a username with leading and trailing spaces such as space hacklarr space in the username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter space followed by hacklarr followed by space in the username textbox
+Enter space followed by Icstunnel1 followed by space in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Authentication fails and the application remains on the login page with a visible sign-in failure message indicating invalid credentials.</t>
+          <t>Application processes the submitted credentials. If the system trims leading and trailing whitespace, login succeeds and the user is redirected to http://172.21.166.115/washtabui/home; otherwise authentication fails and the user remains on the login page with a visible failure indication.</t>
         </is>
       </c>
     </row>
@@ -937,7 +931,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify login attempt with whitespace-only username</t>
+          <t>Verify login fails when username contains only whitespace characters</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -953,15 +947,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter only spaces into the username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter multiple spaces in the username textbox
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Login attempt fails, the application remains on the login page, and visible feedback indicates invalid or missing username.</t>
+          <t>Authentication is rejected and the login page remains visible. A visible login failure or validation indication appears and the application does not redirect to the home page.</t>
         </is>
       </c>
     </row>
@@ -973,7 +967,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify login attempt with whitespace-only password</t>
+          <t>Verify login fails when password contains only whitespace characters</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -989,15 +983,15 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr in username textbox
-Enter only spaces in password textbox
+          <t>Navigate to the login page
+Enter hacklarr in the username textbox
+Enter multiple spaces in the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Authentication fails and the login page remains displayed with a visible sign-in failure message indicating invalid credentials.</t>
+          <t>Authentication attempt fails and the user remains on the login page. A visible authentication failure message or indication is displayed and the browser does not navigate to the home page.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1003,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify behavior when SIGN IN button is clicked multiple times rapidly</t>
+          <t>Verify system behavior when SIGN IN button is clicked repeatedly with valid credentials</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1025,15 +1019,15 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr in username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter hacklarr in the username textbox
+Enter Icstunnel1 in the password textbox
 Click the SIGN IN button multiple times rapidly</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Only one authentication request is processed and the user is redirected once to the home page without duplicate navigation or UI errors.</t>
+          <t>Application processes the login request once and redirects to the home page. Only a single successful navigation to http://172.21.166.115/washtabui/home occurs and no duplicate navigation or visible error appears.</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1039,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify login attempt with extremely long username input</t>
+          <t>Verify login using credentials pasted into username and password fields</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1061,15 +1055,15 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter a very long string exceeding normal username length into the username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Copy hacklarr and paste it into the username textbox
+Copy Icstunnel1 and paste it into the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>The application handles the long input without UI crash, authentication fails, and the user remains on the login page with a visible sign-in failure message.</t>
+          <t>Pasted values are accepted in both fields and authentication succeeds. User is redirected to the home page and the browser URL becomes http://172.21.166.115/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -1081,12 +1075,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Verify login fails with special characters in username</t>
+          <t>Verify login fails when extremely long text values are entered in username and password fields</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1097,15 +1091,15 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter special characters such as @@@### in the username textbox
-Enter Icstunnel1 in password textbox
+          <t>Navigate to the login page
+Enter a very long string exceeding typical username length into the username textbox
+Enter a very long string exceeding typical password length into the password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Authentication fails and the application remains on the login page with a visible error or sign-in failure message indicating invalid credentials.</t>
+          <t>Authentication does not succeed and the application remains stable on the login page without crashes. Browser does not redirect to the home page and the login form remains visible.</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1111,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Verify login submission using Enter key</t>
+          <t>Verify login behavior when credentials are entered with different letter casing</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1133,51 +1127,15 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter hacklarr in username textbox
-Enter Icstunnel1 in password textbox
-Press the Enter key on the keyboard</t>
+          <t>Navigate to the login page
+Enter HACKLARR in the username textbox
+Enter ICSTUNNEL1 in the password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The login form is submitted using the Enter key and the user is redirected to the home page indicating successful authentication.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>WT-LOGIN20</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Verify login attempt with uppercase username</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Open the login page
-Enter HACKLARR in username textbox
-Enter Icstunnel1 in password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Authentication fails and the application remains on the login page with a visible sign-in failure message indicating invalid credentials.</t>
+          <t>If authentication is case sensitive, the login attempt fails and the user remains on the login page with a visible authentication failure indication and no redirect to the home page.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 48
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads and all required UI elements are visible</t>
+          <t>Verify login page loads with username textbox, password textbox, SIGN IN button, home navigation button and back navigation button visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,13 +486,13 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open a browser and navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page layout and visible controls</t>
+          <t>Open browser and navigate to http://172.21.166.115/washtabui/login?data=undefined
+Observe the login page layout and available controls</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads successfully with URL http://172.21.166.115/washtabui/login?data=undefined and the username textbox, password textbox, SIGN IN button, home navigation button, and back navigation button are visible and interactable.</t>
+          <t>Login page loads successfully at URL http://172.21.166.115/washtabui/login?data=undefined and username textbox, password textbox, SIGN IN button, home navigation button and back navigation button are visible and interactable</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify successful login using valid credentials via SIGN IN button</t>
+          <t>Verify successful login using valid username and valid password through SIGN IN button</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,14 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in the username textbox
-Enter Icstunnel1 in the password textbox
+Enter hacklarr into username textbox
+Enter Icstunnel1 into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User is authenticated successfully and the application redirects to the home page. Browser URL changes to http://172.21.166.115/washtabui/home and login page elements are no longer visible.</t>
+          <t>User is authenticated successfully and browser redirects to home page with URL http://172.21.166.115/washtabui/home and login page elements are no longer displayed</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify login submission using keyboard Enter key after entering valid credentials</t>
+          <t>Verify login submission using Enter key from password textbox with valid credentials</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -557,14 +557,14 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in the username textbox
-Enter Icstunnel1 in the password textbox
-Press Enter on the keyboard while the cursor focus is inside the password textbox</t>
+Enter hacklarr into username textbox
+Enter Icstunnel1 into password textbox
+Press Enter key while focus is inside the password textbox</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Login form is submitted through the keyboard action and the application redirects to the home page with URL http://172.21.166.115/washtabui/home indicating successful authentication.</t>
+          <t>Form submission is triggered by Enter key and user is authenticated successfully and redirected to http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with valid username and incorrect password</t>
+          <t>Verify login fails when valid username is used with incorrect password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,14 +593,14 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in the username textbox
-Enter Icstunnel2 in the password textbox
+Enter hacklarr into username textbox
+Enter IncorrectPass123 into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication fails and the user remains on the login page with URL http://172.21.166.115/washtabui/login?data=undefined. A visible sign-in failure or error indication is displayed and the application does not navigate to the home page.</t>
+          <t>Authentication is rejected, a visible sign-in failure message is displayed and the page remains at URL http://172.21.166.115/washtabui/login?data=undefined without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify login fails with invalid username and valid password</t>
+          <t>Verify login fails when invalid username is used with valid password</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -629,14 +629,14 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr123 in the username textbox
-Enter Icstunnel1 in the password textbox
+Enter invaliduser into username textbox
+Enter Icstunnel1 into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication is rejected and the application remains on the login page. Browser URL does not change to the home page and a visible login failure indication appears.</t>
+          <t>Authentication fails, a visible sign-in failure message is displayed and user remains on login page URL http://172.21.166.115/washtabui/login?data=undefined</t>
         </is>
       </c>
     </row>
@@ -665,14 +665,14 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter invaliduser in the username textbox
-Enter invalidpass in the password textbox
+Enter wronguser into username textbox
+Enter wrongpassword into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>System rejects the authentication attempt and the login page remains visible. Browser URL remains the login URL and a visible authentication failure indication is displayed.</t>
+          <t>Authentication attempt is rejected, a sign-in failure message is displayed and the page remains on the login URL without navigation to the home page</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify login attempt when username is empty and password is provided</t>
+          <t>Verify login validation when both username and password fields are empty</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -701,14 +701,14 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Leave the username textbox empty
-Enter Icstunnel1 in the password textbox
+Leave username textbox empty
+Leave password textbox empty
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication does not succeed and the application remains on the login page with a visible validation or authentication failure indication. No navigation to the home page occurs.</t>
+          <t>Login is rejected and the user remains on the login page with a visible validation or authentication failure message and no redirect to the home page</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login attempt when password is empty and username is provided</t>
+          <t>Verify login validation when username is entered and password field is empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -737,14 +737,14 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in the username textbox
-Leave the password textbox empty
+Enter hacklarr into username textbox
+Leave password textbox empty
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication is rejected and the user remains on the login page. A visible validation or authentication failure indication appears and the browser does not redirect to the home page.</t>
+          <t>Login submission is rejected, validation or authentication failure message is displayed and the application remains on login page URL http://172.21.166.115/washtabui/login?data=undefined</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify login attempt when both username and password fields are empty</t>
+          <t>Verify login validation when password is entered and username field is empty</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -773,14 +773,14 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Leave the username textbox empty
-Leave the password textbox empty
+Leave username textbox empty
+Enter Icstunnel1 into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Login submission is rejected and the login page remains visible with a validation or authentication failure indication. Browser does not navigate to the home page.</t>
+          <t>Authentication is not performed, a validation or failure message is displayed and the page remains at login URL</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify password textbox masks entered characters</t>
+          <t>Verify password textbox masks characters while user types password</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -810,12 +810,12 @@
         <is>
           <t>Navigate to the login page
 Click inside the password textbox
-Type Icstunnel1 into the password textbox</t>
+Type Icstunnel1 into password textbox</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Password characters are not displayed as plain text. Each entered character appears masked (for example as dots or asterisks) confirming the field behaves as a password field.</t>
+          <t>Password characters appear masked such as dots or asterisks and the actual password text is not visible on the screen</t>
         </is>
       </c>
     </row>
@@ -827,12 +827,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify navigation to home page using home navigation button from login page</t>
+          <t>Verify login succeeds when valid credentials are entered with leading and trailing spaces</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -844,12 +844,14 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Click the home navigation button</t>
+Enter space hacklarr space into username textbox
+Enter space Icstunnel1 space into password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Application navigates away from the login page and loads the home page. Browser URL becomes http://172.21.166.115/washtabui/home.</t>
+          <t>Application trims leading and trailing spaces, authenticates the user successfully and redirects to http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -861,12 +863,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify navigation to home page using back navigation button from login page</t>
+          <t>Verify login fails when username and password contain only whitespace characters</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -878,12 +880,14 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Click the back navigation button</t>
+Enter multiple spaces into username textbox
+Enter multiple spaces into password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Application navigates away from the login page and loads the home page. Browser URL changes to http://172.21.166.115/washtabui/home.</t>
+          <t>Login attempt is rejected, visible validation or sign-in failure message appears and browser remains on the login page URL</t>
         </is>
       </c>
     </row>
@@ -895,7 +899,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login behavior when credentials contain leading and trailing whitespace</t>
+          <t>Verify login using copy and paste actions for username and password fields</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -911,15 +915,16 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter space followed by hacklarr followed by space in the username textbox
-Enter space followed by Icstunnel1 followed by space in the password textbox
+          <t>Copy text hacklarr to clipboard
+Paste the copied value into username textbox
+Copy text Icstunnel1 to clipboard
+Paste the copied value into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Application processes the submitted credentials. If the system trims leading and trailing whitespace, login succeeds and the user is redirected to http://172.21.166.115/washtabui/home; otherwise authentication fails and the user remains on the login page with a visible failure indication.</t>
+          <t>Pasted values are accepted correctly and user is authenticated successfully and redirected to home page URL http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -931,12 +936,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify login fails when username contains only whitespace characters</t>
+          <t>Verify system behavior when SIGN IN button is clicked repeatedly during login submission</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -948,14 +953,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter multiple spaces in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
+Enter hacklarr into username textbox
+Enter Icstunnel1 into password textbox
+Rapidly click the SIGN IN button multiple times</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Authentication is rejected and the login page remains visible. A visible login failure or validation indication appears and the application does not redirect to the home page.</t>
+          <t>Application processes only a single authentication request and redirects once to the home page without duplicate navigation, duplicate sessions or visible errors</t>
         </is>
       </c>
     </row>
@@ -967,12 +972,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify login fails when password contains only whitespace characters</t>
+          <t>Verify navigation to home page using home navigation button from login page</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -984,14 +989,12 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in the username textbox
-Enter multiple spaces in the password textbox
-Click the SIGN IN button</t>
+Click the home navigation button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Authentication attempt fails and the user remains on the login page. A visible authentication failure message or indication is displayed and the browser does not navigate to the home page.</t>
+          <t>Browser navigates directly to home page and URL becomes http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -1003,12 +1006,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify system behavior when SIGN IN button is clicked repeatedly with valid credentials</t>
+          <t>Verify navigation to home page using back navigation button from login page</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1020,14 +1023,12 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button multiple times rapidly</t>
+Click the back navigation button</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Application processes the login request once and redirects to the home page. Only a single successful navigation to http://172.21.166.115/washtabui/home occurs and no duplicate navigation or visible error appears.</t>
+          <t>Application navigates away from the login page and browser URL becomes http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1040,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify login using credentials pasted into username and password fields</t>
+          <t>Verify login behavior when extremely long username and password values are entered</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1056,14 +1057,14 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Copy hacklarr and paste it into the username textbox
-Copy Icstunnel1 and paste it into the password textbox
+Enter a string longer than 200 characters into username textbox
+Enter a string longer than 200 characters into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pasted values are accepted in both fields and authentication succeeds. User is redirected to the home page and the browser URL becomes http://172.21.166.115/washtabui/home.</t>
+          <t>Authentication attempt fails safely without page crash or layout break and the login page remains visible with a sign-in failure message</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1076,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Verify login fails when extremely long text values are entered in username and password fields</t>
+          <t>Verify login fails when username case differs from the valid credential case</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1092,50 +1093,14 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter a very long string exceeding typical username length into the username textbox
-Enter a very long string exceeding typical password length into the password textbox
+Enter HACKLARR into username textbox
+Enter Icstunnel1 into password textbox
 Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Authentication does not succeed and the application remains stable on the login page without crashes. Browser does not redirect to the home page and the login form remains visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WT-LOGIN19</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Verify login behavior when credentials are entered with different letter casing</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Navigate to the login page
-Enter HACKLARR in the username textbox
-Enter ICSTUNNEL1 in the password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>If authentication is case sensitive, the login attempt fails and the user remains on the login page with a visible authentication failure indication and no redirect to the home page.</t>
+          <t>Authentication fails due to username case mismatch and a sign-in failure message is displayed while the browser remains on the login page</t>
         </is>
       </c>
     </row>

</xml_diff>